<commit_message>
Cập nhật: 16/09/2026 18:21
</commit_message>
<xml_diff>
--- a/templates/mau.xlsx
+++ b/templates/mau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhuan\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6363AB64-B037-4E43-A3A6-3FD3E342AD04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A1A60A1-8767-49B3-9EA2-54EDC5B16BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -607,7 +607,7 @@
     <col min="11" max="11" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
         <v>37</v>
       </c>
@@ -1378,9 +1378,6 @@
       <c r="K38" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
   <dataValidations count="6">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" errorTitle="Dữ liệu không hợp lệ" error="Chỉ được nhập số nguyên không âm." sqref="C19:F38" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>

</xml_diff>